<commit_message>
Asistan test seti: 20 soru ve sonuçlar
</commit_message>
<xml_diff>
--- a/docs/asistan_test_seti.xlsx
+++ b/docs/asistan_test_seti.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ECEM\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F13727B-59D9-4FE8-B41D-4D2AD847D0E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DDC8EC0-FC22-4378-9CB0-6F00EFD87FB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="828" yWindow="2268" windowWidth="22260" windowHeight="10692" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Seti" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="101">
   <si>
     <t>Soru No</t>
   </si>
@@ -58,9 +58,6 @@
   </si>
   <si>
     <t>Kaynak gösterdi mi?</t>
-  </si>
-  <si>
-    <t>Not / Düzeltme</t>
   </si>
   <si>
     <t>Yangında asansör kullanılır mı?</t>
@@ -366,6 +363,12 @@
   <si>
     <t xml:space="preserve">Bu konu bilgi tabanında kayıtlı değil, itfaiyenin talimatına uyun. Acil durum numarası 112'dir.
 </t>
+  </si>
+  <si>
+    <t>Evet</t>
+  </si>
+  <si>
+    <t>Hayır</t>
   </si>
 </sst>
 </file>
@@ -773,7 +776,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -786,7 +789,7 @@
     <col min="9" max="9" width="32" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -811,469 +814,526 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:8" ht="23.85" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" ht="23.85" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="2">
-        <v>1</v>
-      </c>
-      <c r="B2" s="3" t="s">
+      <c r="C2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="3" t="s">
-        <v>12</v>
-      </c>
       <c r="F2" s="12" t="s">
-        <v>83</v>
-      </c>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-    </row>
-    <row r="3" spans="1:9" ht="23.85" customHeight="1" x14ac:dyDescent="0.3">
+        <v>82</v>
+      </c>
+      <c r="G2" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="23.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>2</v>
       </c>
       <c r="B3" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="3" t="s">
-        <v>15</v>
-      </c>
       <c r="F3" s="12" t="s">
-        <v>84</v>
-      </c>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
-    </row>
-    <row r="4" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+        <v>83</v>
+      </c>
+      <c r="G3" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>3</v>
       </c>
       <c r="B4" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E4" s="3" t="s">
-        <v>18</v>
-      </c>
       <c r="F4" s="12" t="s">
-        <v>85</v>
-      </c>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
-    </row>
-    <row r="5" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+        <v>84</v>
+      </c>
+      <c r="G4" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>4</v>
       </c>
       <c r="B5" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="E5" s="3" t="s">
-        <v>22</v>
-      </c>
       <c r="F5" s="12" t="s">
-        <v>86</v>
-      </c>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
-    </row>
-    <row r="6" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+        <v>85</v>
+      </c>
+      <c r="G5" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>5</v>
       </c>
       <c r="B6" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C6" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6" s="3" t="s">
+      <c r="E6" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="3" t="s">
-        <v>25</v>
-      </c>
       <c r="F6" s="12" t="s">
-        <v>87</v>
-      </c>
-      <c r="G6" s="4"/>
-      <c r="H6" s="4"/>
-      <c r="I6" s="4"/>
-    </row>
-    <row r="7" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+        <v>86</v>
+      </c>
+      <c r="G6" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>6</v>
       </c>
       <c r="B7" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D7" s="3" t="s">
+      <c r="E7" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="E7" s="3" t="s">
-        <v>28</v>
-      </c>
       <c r="F7" s="12" t="s">
-        <v>88</v>
-      </c>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4"/>
-      <c r="I7" s="4"/>
-    </row>
-    <row r="8" spans="1:9" ht="23.85" customHeight="1" x14ac:dyDescent="0.3">
+        <v>87</v>
+      </c>
+      <c r="G7" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="23.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>7</v>
       </c>
       <c r="B8" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C8" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D8" s="3" t="s">
+      <c r="E8" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="E8" s="3" t="s">
-        <v>31</v>
-      </c>
       <c r="F8" s="12" t="s">
-        <v>89</v>
-      </c>
-      <c r="G8" s="4"/>
-      <c r="H8" s="4"/>
-      <c r="I8" s="4"/>
-    </row>
-    <row r="9" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+        <v>88</v>
+      </c>
+      <c r="G8" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
         <v>8</v>
       </c>
       <c r="B9" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D9" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D9" s="3" t="s">
+      <c r="E9" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="E9" s="3" t="s">
-        <v>34</v>
-      </c>
       <c r="F9" s="12" t="s">
-        <v>90</v>
-      </c>
-      <c r="G9" s="4"/>
-      <c r="H9" s="4"/>
-      <c r="I9" s="4"/>
-    </row>
-    <row r="10" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+        <v>89</v>
+      </c>
+      <c r="G9" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
         <v>9</v>
       </c>
       <c r="B10" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C10" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D10" s="3" t="s">
+      <c r="E10" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="E10" s="3" t="s">
-        <v>37</v>
-      </c>
       <c r="F10" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="G10" s="4"/>
-      <c r="H10" s="4"/>
-      <c r="I10" s="4"/>
-    </row>
-    <row r="11" spans="1:9" ht="23.85" customHeight="1" x14ac:dyDescent="0.3">
+        <v>90</v>
+      </c>
+      <c r="G10" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="23.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
         <v>10</v>
       </c>
       <c r="B11" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C11" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D11" s="3" t="s">
+      <c r="E11" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="E11" s="3" t="s">
-        <v>40</v>
-      </c>
       <c r="F11" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="G11" s="4"/>
-      <c r="H11" s="4"/>
-      <c r="I11" s="4"/>
-    </row>
-    <row r="12" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+        <v>91</v>
+      </c>
+      <c r="G11" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
         <v>11</v>
       </c>
       <c r="B12" s="13" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D12" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="C12" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D12" s="3" t="s">
+      <c r="E12" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="E12" s="3" t="s">
-        <v>43</v>
-      </c>
       <c r="F12" s="12" t="s">
-        <v>93</v>
-      </c>
-      <c r="G12" s="4"/>
-      <c r="H12" s="4"/>
-      <c r="I12" s="4"/>
-    </row>
-    <row r="13" spans="1:9" ht="23.85" customHeight="1" x14ac:dyDescent="0.3">
+        <v>92</v>
+      </c>
+      <c r="G12" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="23.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2">
         <v>12</v>
       </c>
       <c r="B13" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D13" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C13" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D13" s="3" t="s">
+      <c r="E13" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="E13" s="3" t="s">
-        <v>46</v>
-      </c>
       <c r="F13" s="12" t="s">
-        <v>94</v>
-      </c>
-      <c r="G13" s="4"/>
-      <c r="H13" s="4"/>
-      <c r="I13" s="4"/>
-    </row>
-    <row r="14" spans="1:9" ht="23.85" customHeight="1" x14ac:dyDescent="0.3">
+        <v>93</v>
+      </c>
+      <c r="G13" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="23.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2">
         <v>13</v>
       </c>
       <c r="B14" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D14" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C14" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D14" s="3" t="s">
+      <c r="E14" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="E14" s="3" t="s">
-        <v>49</v>
-      </c>
       <c r="F14" s="12" t="s">
-        <v>95</v>
-      </c>
-      <c r="G14" s="4"/>
-      <c r="H14" s="4"/>
-      <c r="I14" s="4"/>
-    </row>
-    <row r="15" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+        <v>94</v>
+      </c>
+      <c r="G14" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2">
         <v>14</v>
       </c>
       <c r="B15" s="13" t="s">
+        <v>49</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D15" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="C15" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D15" s="3" t="s">
+      <c r="E15" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="E15" s="3" t="s">
-        <v>52</v>
-      </c>
       <c r="F15" s="12" t="s">
-        <v>96</v>
-      </c>
-      <c r="G15" s="4"/>
-      <c r="H15" s="4"/>
-      <c r="I15" s="4"/>
-    </row>
-    <row r="16" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+        <v>95</v>
+      </c>
+      <c r="G15" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2">
         <v>15</v>
       </c>
       <c r="B16" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D16" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="C16" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D16" s="3" t="s">
+      <c r="E16" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="E16" s="3" t="s">
-        <v>55</v>
-      </c>
       <c r="F16" s="12" t="s">
-        <v>97</v>
-      </c>
-      <c r="G16" s="4"/>
-      <c r="H16" s="4"/>
-      <c r="I16" s="4"/>
-    </row>
-    <row r="17" spans="1:9" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>96</v>
+      </c>
+      <c r="G16" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="5">
         <v>16</v>
       </c>
       <c r="B17" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="C17" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="D17" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="D17" s="6" t="s">
+      <c r="E17" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="E17" s="6" t="s">
-        <v>59</v>
-      </c>
       <c r="F17" s="12" t="s">
-        <v>98</v>
-      </c>
-      <c r="G17" s="4"/>
-      <c r="H17" s="4"/>
-      <c r="I17" s="4"/>
-    </row>
-    <row r="18" spans="1:9" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>97</v>
+      </c>
+      <c r="G17" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H17" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="5">
         <v>17</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C18" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="D18" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="D18" s="6" t="s">
+      <c r="E18" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="E18" s="6" t="s">
-        <v>59</v>
-      </c>
       <c r="F18" s="12" t="s">
-        <v>98</v>
-      </c>
-      <c r="G18" s="4"/>
-      <c r="H18" s="4"/>
-      <c r="I18" s="4"/>
-    </row>
-    <row r="19" spans="1:9" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>97</v>
+      </c>
+      <c r="G18" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H18" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="5">
         <v>18</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C19" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="D19" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="D19" s="6" t="s">
+      <c r="E19" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="E19" s="6" t="s">
-        <v>59</v>
-      </c>
       <c r="F19" s="12" t="s">
-        <v>99</v>
-      </c>
-      <c r="G19" s="4"/>
-      <c r="H19" s="4"/>
-      <c r="I19" s="4"/>
-    </row>
-    <row r="20" spans="1:9" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>98</v>
+      </c>
+      <c r="G19" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H19" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="5">
         <v>19</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C20" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="D20" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="D20" s="6" t="s">
+      <c r="E20" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="E20" s="6" t="s">
-        <v>59</v>
-      </c>
       <c r="F20" s="12" t="s">
-        <v>98</v>
-      </c>
-      <c r="G20" s="4"/>
-      <c r="H20" s="4"/>
-      <c r="I20" s="4"/>
-    </row>
-    <row r="21" spans="1:9" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>97</v>
+      </c>
+      <c r="G20" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H20" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="5">
         <v>20</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C21" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="D21" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="D21" s="6" t="s">
+      <c r="E21" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="E21" s="6" t="s">
-        <v>59</v>
-      </c>
       <c r="F21" s="12" t="s">
-        <v>98</v>
-      </c>
-      <c r="G21" s="4"/>
-      <c r="H21" s="4"/>
-      <c r="I21" s="4"/>
+        <v>97</v>
+      </c>
+      <c r="G21" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>100</v>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="2">
@@ -1302,12 +1362,12 @@
   <sheetData>
     <row r="1" spans="1:2" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B2" s="8">
         <f>COUNTA('Test Seti'!B2:B21)</f>
@@ -1316,7 +1376,7 @@
     </row>
     <row r="3" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="8" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B3" s="8">
         <f>COUNTIF('Test Seti'!C2:C21,"Bilgi tabanında VAR")</f>
@@ -1325,7 +1385,7 @@
     </row>
     <row r="4" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B4" s="8">
         <f>COUNTIF('Test Seti'!C2:C21,"Bilgi tabanında YOK")</f>
@@ -1334,7 +1394,7 @@
     </row>
     <row r="5" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B5">
         <f>COUNTIF('Test Seti'!C2:C21,"Tuzak (bilgi tabanında VAR)")</f>
@@ -1343,16 +1403,16 @@
     </row>
     <row r="6" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B6" s="8">
         <f>COUNTIF('Test Seti'!G2:G21,"Doğru")</f>
-        <v>0</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B7" s="8">
         <f>COUNTIF('Test Seti'!G2:G21,"Yanlış")</f>
@@ -1361,7 +1421,7 @@
     </row>
     <row r="8" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B8" s="8">
         <f>COUNTIF('Test Seti'!G2:G21,"Uydurma")</f>
@@ -1370,7 +1430,7 @@
     </row>
     <row r="9" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B9" s="8">
         <f>COUNTIF('Test Seti'!G2:G21,"Eksik madde")</f>
@@ -1379,29 +1439,29 @@
     </row>
     <row r="10" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B10" s="8">
         <f>COUNTIF('Test Seti'!H2:H21,"Evet")</f>
-        <v>0</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B11" s="8">
         <f>B2-COUNTA('Test Seti'!G2:G21)</f>
-        <v>20</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="B12" s="9" t="str">
+        <v>74</v>
+      </c>
+      <c r="B12" s="9">
         <f>IF(B2-B11=0,"",B6/(B2-B11))</f>
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1410,42 +1470,42 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B14" s="8" t="str">
         <f>"20 soruda "&amp;B6&amp;" doğru, "&amp;B8&amp;" uydurma (hedef 0), "&amp;B9&amp;" eksik madde."</f>
-        <v>20 soruda 0 doğru, 0 uydurma (hedef 0), 0 eksik madde.</v>
+        <v>20 soruda 20 doğru, 0 uydurma (hedef 0), 0 eksik madde.</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="16" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="11" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="18" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="8" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="19" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="8" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="20" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="8" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
   </sheetData>

</xml_diff>